<commit_message>
fix: map No Registration - Lokasi to reg_lokasi in MIT upload
reg_lokasi was always saved as NULL because MIT_MAPPER had no entry
for the "No Registration - Lokasi" Excel header, and the frontend
whitelist parser dropped the column before it ever reached the
backend. Add the mapping, add the header to expectedHeaders/template,
and add a regression test.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/Template MIT Quartal.xlsx
+++ b/frontend/public/templates/Template MIT Quartal.xlsx
@@ -1,142 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS ZENBOOK\Documents\1. College\Project\3. Pertamina\Template\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48F8D16-8800-44C4-AA92-E997932BF425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" xr2:uid="{0B7EFD56-CD58-CC40-91CF-4D30E8DE81C2}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>MIT Declaration Date</t>
-  </si>
-  <si>
-    <t>MIT Title / Asset</t>
-  </si>
-  <si>
-    <t>Integrity Threats</t>
-  </si>
-  <si>
-    <t>Possible Scenario</t>
-  </si>
-  <si>
-    <t>Consequences</t>
-  </si>
-  <si>
-    <t>Available Safeguard/Control</t>
-  </si>
-  <si>
-    <t>Rec. No.</t>
-  </si>
-  <si>
-    <t>Recommendation / Action</t>
-  </si>
-  <si>
-    <t>PIC</t>
-  </si>
-  <si>
-    <t>Target Closing</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Risk</t>
-  </si>
-  <si>
-    <t>MIT Status</t>
-  </si>
-  <si>
-    <t>Evidence</t>
-  </si>
-  <si>
-    <t>Closing Date</t>
-  </si>
-  <si>
-    <t>No Registration - Jenis MIT</t>
-  </si>
-  <si>
-    <t>No Registration - Kategori</t>
-  </si>
-  <si>
-    <t>No Registration - Tahun</t>
-  </si>
-  <si>
-    <t>No Registration - No</t>
-  </si>
-  <si>
-    <t>Current Risk - Likelihood</t>
-  </si>
-  <si>
-    <t>Current Risk - Severity</t>
-  </si>
-  <si>
-    <t>Current Risk - Risk</t>
-  </si>
-  <si>
-    <t>Target Risk (After implemented Recommendation) - Likelihood</t>
-  </si>
-  <si>
-    <t>Target Risk (After implemented Recommendation) - Severity</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="0"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -174,24 +73,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -511,103 +469,161 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F76B2F-11E0-564D-B111-E3C1876BE770}">
-  <dimension ref="A1:X1"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Y1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="29.796875" customWidth="1"/>
-    <col min="2" max="4" width="29.5" customWidth="1"/>
-    <col min="5" max="5" width="24.296875" customWidth="1"/>
-    <col min="6" max="6" width="17.796875" customWidth="1"/>
-    <col min="7" max="7" width="18.296875" customWidth="1"/>
-    <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="18.69921875" customWidth="1"/>
-    <col min="10" max="10" width="33.19921875" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
-    <col min="12" max="12" width="26.296875" customWidth="1"/>
-    <col min="13" max="13" width="21.69921875" customWidth="1"/>
-    <col min="15" max="15" width="29.796875" customWidth="1"/>
-    <col min="19" max="20" width="34.796875" customWidth="1"/>
-    <col min="22" max="22" width="18.69921875" customWidth="1"/>
-    <col min="24" max="24" width="20.296875" customWidth="1"/>
+    <col width="29.796875" customWidth="1" min="1" max="1"/>
+    <col width="29.796875" customWidth="1" min="2" max="2"/>
+    <col width="29.5" customWidth="1" min="3" max="3"/>
+    <col width="24.296875" customWidth="1" min="6" max="6"/>
+    <col width="17.796875" customWidth="1" min="7" max="7"/>
+    <col width="18.296875" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="18.69921875" customWidth="1" min="10" max="10"/>
+    <col width="33.19921875" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="26.296875" customWidth="1" min="13" max="13"/>
+    <col width="21.69921875" customWidth="1" min="14" max="14"/>
+    <col width="29.796875" customWidth="1" min="16" max="16"/>
+    <col width="34.796875" customWidth="1" min="20" max="20"/>
+    <col width="18.69921875" customWidth="1" min="23" max="23"/>
+    <col width="20.296875" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>14</v>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No Registration - Lokasi</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>No Registration - Jenis MIT</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>No Registration - Kategori</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>No Registration - Tahun</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>No Registration - No</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MIT Declaration Date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MIT Title / Asset</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Integrity Threats</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Possible Scenario</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Available Safeguard/Control</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Current Risk - Likelihood</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Current Risk - Severity</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Current Risk - Risk</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Rec. No.</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Recommendation / Action</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>PIC</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Target Closing</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Target Risk (After implemented Recommendation) - Likelihood</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Target Risk (After implemented Recommendation) - Severity</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>MIT Status</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Closing Date</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: harden Data Gathering uploads against silently lost or wrong data
- Excel dates were shifted one day back in WIB (toISOString); format in local time
- MIT: Lokasi comes from the field dropdown, removed from template and header check
- MIT: target_closing is free text now (TAR 2027, TBC, Q4 2025 were saved as NULL)
- MIT: validate No Registration, status, declaration date and Risk = L x S
- all modules: flag date cells the backend cannot parse instead of storing NULL
- detect the header row below title rows; keep case-distinct HAZOP Rec. No. columns apart
- backend: parse Excel serial dates and day-fraction times (Zona PSE List)
- widen HAZID/HAZOP category and LOPA final_element, which truncated real sheets
</commit_message>
<xml_diff>
--- a/frontend/public/templates/Template MIT Quartal.xlsx
+++ b/frontend/public/templates/Template MIT Quartal.xlsx
@@ -474,149 +474,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
     <col width="29.796875" customWidth="1" min="1" max="1"/>
-    <col width="29.796875" customWidth="1" min="2" max="2"/>
+    <col width="29.5" customWidth="1" min="2" max="2"/>
     <col width="29.5" customWidth="1" min="3" max="3"/>
-    <col width="24.296875" customWidth="1" min="6" max="6"/>
-    <col width="17.796875" customWidth="1" min="7" max="7"/>
-    <col width="18.296875" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="18.69921875" customWidth="1" min="10" max="10"/>
-    <col width="33.19921875" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="26.296875" customWidth="1" min="13" max="13"/>
+    <col width="24.296875" customWidth="1" min="5" max="5"/>
+    <col width="17.796875" customWidth="1" min="6" max="6"/>
+    <col width="18.296875" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="18.69921875" customWidth="1" min="9" max="9"/>
+    <col width="33.19921875" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="26.296875" customWidth="1" min="12" max="12"/>
+    <col width="21.69921875" customWidth="1" min="13" max="13"/>
     <col width="21.69921875" customWidth="1" min="14" max="14"/>
+    <col width="29.796875" customWidth="1" min="15" max="15"/>
     <col width="29.796875" customWidth="1" min="16" max="16"/>
+    <col width="34.796875" customWidth="1" min="19" max="19"/>
     <col width="34.796875" customWidth="1" min="20" max="20"/>
+    <col width="18.69921875" customWidth="1" min="22" max="22"/>
     <col width="18.69921875" customWidth="1" min="23" max="23"/>
+    <col width="20.296875" customWidth="1" min="24" max="24"/>
     <col width="20.296875" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>No Registration - Lokasi</t>
+          <t>No Registration - Jenis MIT</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>No Registration - Jenis MIT</t>
+          <t>No Registration - Kategori</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>No Registration - Kategori</t>
+          <t>No Registration - Tahun</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>No Registration - Tahun</t>
+          <t>No Registration - No</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>No Registration - No</t>
+          <t>MIT Declaration Date</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>MIT Declaration Date</t>
+          <t>MIT Title / Asset</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>MIT Title / Asset</t>
+          <t>Integrity Threats</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Integrity Threats</t>
+          <t>Possible Scenario</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Possible Scenario</t>
+          <t>Consequences</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Consequences</t>
+          <t>Available Safeguard/Control</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Available Safeguard/Control</t>
+          <t>Current Risk - Likelihood</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Current Risk - Likelihood</t>
+          <t>Current Risk - Severity</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Current Risk - Severity</t>
+          <t>Current Risk - Risk</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Current Risk - Risk</t>
+          <t>Rec. No.</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Rec. No.</t>
+          <t>Recommendation / Action</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Recommendation / Action</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>PIC</t>
+          <t>Target Closing</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Target Closing</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Target Risk (After implemented Recommendation) - Likelihood</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Target Risk (After implemented Recommendation) - Likelihood</t>
+          <t>Target Risk (After implemented Recommendation) - Severity</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Target Risk (After implemented Recommendation) - Severity</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>MIT Status</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>MIT Status</t>
+          <t>Evidence</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Closing Date</t>
         </is>

</xml_diff>